<commit_message>
Add PWRBCK techs to BAU/INV/OPT and enable ELC*02 remap
Introduces Z_TEMP_add_pwrbck_to_scenarios.py, a one-shot upsert that
writes the 19 PWRBCK* rows from OG_csvs_inputs into Secondary Techs,
VariableCost, Fixed Horizon Parameters, Model Base Year Secondary and
Projections Secondary across the three scenarios, sobrescribiendo en
sitio sin tocar filas no-PWRBCK. Activa también la flag
pwrbck_output_to_elc02 (Config_region_consolidation.yaml) y aplica el
remap correspondiente: las BCK ahora producen ELC{ISO3}XX02 en lugar
de ELC{ISO3}XX01. Refleja el cambio en los 9 Excel de A1_Outputs.
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -30961,12 +30961,12 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>ELCARGXX01</t>
+          <t>ELCARGXX02</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>Electricity, Argentina, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Argentina, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J529" t="n">
@@ -30989,12 +30989,12 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>ELCBOLXX01</t>
+          <t>ELCBOLXX02</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>Electricity, Bolivia, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Bolivia, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J530" t="n">
@@ -31017,12 +31017,12 @@
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>ELCBRAXX01</t>
+          <t>ELCBRAXX02</t>
         </is>
       </c>
       <c r="I531" t="inlineStr">
         <is>
-          <t>Electricity, Brazil, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Brazil, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J531" t="n">
@@ -31045,12 +31045,12 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>ELCBRBXX01</t>
+          <t>ELCBRBXX02</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
         <is>
-          <t>Electricity, Barbados, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Barbados, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J532" t="n">
@@ -31073,12 +31073,12 @@
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>ELCCHLXX01</t>
+          <t>ELCCHLXX02</t>
         </is>
       </c>
       <c r="I533" t="inlineStr">
         <is>
-          <t>Electricity, Chile, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Chile, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J533" t="n">
@@ -31101,12 +31101,12 @@
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>ELCCOLXX01</t>
+          <t>ELCCOLXX02</t>
         </is>
       </c>
       <c r="I534" t="inlineStr">
         <is>
-          <t>Electricity, Colombia, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Colombia, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J534" t="n">
@@ -31129,12 +31129,12 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>ELCCRIXX01</t>
+          <t>ELCCRIXX02</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
         <is>
-          <t>Electricity, Costa Rica, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Costa Rica, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J535" t="n">
@@ -31157,12 +31157,12 @@
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>ELCDOMXX01</t>
+          <t>ELCDOMXX02</t>
         </is>
       </c>
       <c r="I536" t="inlineStr">
         <is>
-          <t>Electricity, Dominican Republic, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Dominican Republic, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J536" t="n">
@@ -31185,12 +31185,12 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>ELCECUXX01</t>
+          <t>ELCECUXX02</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>Electricity, Ecuador, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Ecuador, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J537" t="n">
@@ -31213,12 +31213,12 @@
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>ELCGTMXX01</t>
+          <t>ELCGTMXX02</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
         <is>
-          <t>Electricity, Guatemala, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Guatemala, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J538" t="n">
@@ -31241,12 +31241,12 @@
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>ELCHNDXX01</t>
+          <t>ELCHNDXX02</t>
         </is>
       </c>
       <c r="I539" t="inlineStr">
         <is>
-          <t>Electricity, Honduras, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Honduras, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J539" t="n">
@@ -31269,12 +31269,12 @@
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>ELCHTIXX01</t>
+          <t>ELCHTIXX02</t>
         </is>
       </c>
       <c r="I540" t="inlineStr">
         <is>
-          <t>Electricity, Haiti, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Haiti, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J540" t="n">
@@ -31297,12 +31297,12 @@
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>ELCMEXXX01</t>
+          <t>ELCMEXXX02</t>
         </is>
       </c>
       <c r="I541" t="inlineStr">
         <is>
-          <t>Electricity, Mexico, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Mexico, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J541" t="n">
@@ -31325,12 +31325,12 @@
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>ELCNICXX01</t>
+          <t>ELCNICXX02</t>
         </is>
       </c>
       <c r="I542" t="inlineStr">
         <is>
-          <t>Electricity, Nicaragua, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Nicaragua, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J542" t="n">
@@ -31353,12 +31353,12 @@
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>ELCPANXX01</t>
+          <t>ELCPANXX02</t>
         </is>
       </c>
       <c r="I543" t="inlineStr">
         <is>
-          <t>Electricity, Panama, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Panama, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J543" t="n">
@@ -31381,12 +31381,12 @@
       </c>
       <c r="H544" t="inlineStr">
         <is>
-          <t>ELCPERXX01</t>
+          <t>ELCPERXX02</t>
         </is>
       </c>
       <c r="I544" t="inlineStr">
         <is>
-          <t>Electricity, Peru, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Peru, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J544" t="n">
@@ -31409,12 +31409,12 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>ELCPRYXX01</t>
+          <t>ELCPRYXX02</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
         <is>
-          <t>Electricity, Paraguay, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Paraguay, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J545" t="n">
@@ -31437,12 +31437,12 @@
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>ELCSLVXX01</t>
+          <t>ELCSLVXX02</t>
         </is>
       </c>
       <c r="I546" t="inlineStr">
         <is>
-          <t>Electricity, El Salvador, Region XX, NO renewable power plant output</t>
+          <t>Electricity, El Salvador, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J546" t="n">
@@ -31465,12 +31465,12 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>ELCURYXX01</t>
+          <t>ELCURYXX02</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
         <is>
-          <t>Electricity, Uruguay, Region XX, NO renewable power plant output</t>
+          <t>Electricity, Uruguay, region XX, transmission line output</t>
         </is>
       </c>
       <c r="J547" t="n">

</xml_diff>

<commit_message>
feat(A1): IAR de transmision por pais en archivos AR (Demand Techs)
Nuevo script Z_AUX_update_transmission_iar.py que fija el Input Activity
Ratio de las 114 tecnologias de transmision (6 prefijos x 19 paises) en la
hoja 'Demand Techs' de los archivos AR, preservando formato.

- Base_Year: Value.Fuel.I = IAR por tech.
- Projections: IAR en 2023-2050 solo en filas Direction=Input (Output intacto).
- Mapeo: PWRTRN/TRNNLI->No-Renovable, RNWTRN/RNWNLI->Renovable,
  RNWRPO/TRNRPO->Repotenciada; pais = tech[6:9].
- Aplicado a los 4 escenarios (BAU/INV/OPT/VGB): 13224 celdas.
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -33702,7 +33702,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -33743,7 +33743,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -33784,7 +33784,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -33825,7 +33825,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>1.005</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -33866,7 +33866,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -33907,7 +33907,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>1.005</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -34030,7 +34030,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -34071,7 +34071,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -34112,7 +34112,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -34153,7 +34153,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -34194,7 +34194,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -34235,7 +34235,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -34358,7 +34358,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>1.037</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -34399,7 +34399,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>1.037</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -34440,7 +34440,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>1.037</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -34481,7 +34481,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -34522,7 +34522,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>1.037</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -34563,7 +34563,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -34686,7 +34686,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -34727,7 +34727,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -34768,7 +34768,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -34809,7 +34809,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -34850,7 +34850,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -34891,7 +34891,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -35014,7 +35014,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -35055,7 +35055,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -35096,7 +35096,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -35137,7 +35137,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -35178,7 +35178,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>1.031</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -35219,7 +35219,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -35342,7 +35342,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>1.034</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -35383,7 +35383,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>1.034</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -35424,7 +35424,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>1.034</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -35465,7 +35465,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -35506,7 +35506,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>1.034</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -35547,7 +35547,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -35670,7 +35670,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -35711,7 +35711,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -35752,7 +35752,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -35793,7 +35793,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -35834,7 +35834,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -35875,7 +35875,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -35998,7 +35998,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -36039,7 +36039,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -36080,7 +36080,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -36121,7 +36121,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>1.013</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -36162,7 +36162,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -36203,7 +36203,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>1.013</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -36326,7 +36326,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>1.018</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -36367,7 +36367,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>1.018</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -36408,7 +36408,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>1.018</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -36449,7 +36449,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1</v>
+        <v>1.009</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -36490,7 +36490,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1</v>
+        <v>1.018</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -36531,7 +36531,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1</v>
+        <v>1.009</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -36654,7 +36654,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -36695,7 +36695,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -36736,7 +36736,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -36777,7 +36777,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -36818,7 +36818,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>1.026</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -36859,7 +36859,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -36982,7 +36982,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -37023,7 +37023,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -37064,7 +37064,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -37105,7 +37105,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -37146,7 +37146,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -37187,7 +37187,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -37310,7 +37310,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -37351,7 +37351,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -37392,7 +37392,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -37433,7 +37433,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -37474,7 +37474,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -37515,7 +37515,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -37638,7 +37638,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -37679,7 +37679,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -37720,7 +37720,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -37761,7 +37761,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>1.013</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -37802,7 +37802,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>1.039</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -37843,7 +37843,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>1</v>
+        <v>1.013</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -37966,7 +37966,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1</v>
+        <v>1.029</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -38007,7 +38007,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>1.029</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -38048,7 +38048,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1</v>
+        <v>1.029</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -38089,7 +38089,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -38130,7 +38130,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>1.029</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -38171,7 +38171,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>1.006</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -38294,7 +38294,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -38335,7 +38335,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -38376,7 +38376,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -38417,7 +38417,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -38458,7 +38458,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1</v>
+        <v>1.033</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -38499,7 +38499,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -38622,7 +38622,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -38663,7 +38663,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -38704,7 +38704,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -38745,7 +38745,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>1.003</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -38786,7 +38786,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>1</v>
+        <v>1.016</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -38827,7 +38827,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>1</v>
+        <v>1.003</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -38950,7 +38950,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -38991,7 +38991,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -39032,7 +39032,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -39073,7 +39073,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>1.012</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -39114,7 +39114,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -39155,7 +39155,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>1</v>
+        <v>1.012</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -39278,7 +39278,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>1</v>
+        <v>1.044</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -39319,7 +39319,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>1</v>
+        <v>1.044</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -39360,7 +39360,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1</v>
+        <v>1.044</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -39401,7 +39401,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>1</v>
+        <v>1.025</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -39442,7 +39442,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>1</v>
+        <v>1.044</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -39483,7 +39483,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>1</v>
+        <v>1.025</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -39606,7 +39606,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -39647,7 +39647,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -39688,7 +39688,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -39729,7 +39729,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>1</v>
+        <v>1.012</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -39770,7 +39770,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
@@ -39811,7 +39811,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>1</v>
+        <v>1.012</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>

</xml_diff>